<commit_message>
edit to sample num qa link in MI 19 file
</commit_message>
<xml_diff>
--- a/data/raw/GLNPO 2024 Spring/GLNPO 2024 Spring/Michigan/D20/Zoops/MI 19 D20 QA Spring 2024 24GM00Q74 Zoop.xlsx
+++ b/data/raw/GLNPO 2024 Spring/GLNPO 2024 Spring/Michigan/D20/Zoops/MI 19 D20 QA Spring 2024 24GM00Q74 Zoop.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmars\OneDrive\Desktop\CCM Work Files\GLNPO Zooplankton Database\data\raw\GLNPO 2024 Spring\GLNPO 2024 Spring\Michigan\D20\Zoops\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAB3CA58-200C-4DA8-B943-827843CAA024}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E274B3DD-CC77-4944-A844-6C2CD9463C46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22D018C6-56D2-4079-B668-5B560F82E708}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{22D018C6-56D2-4079-B668-5B560F82E708}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="13" r:id="rId2"/>
+    <pivotCache cacheId="2" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -257,7 +257,7 @@
     <t>D20</t>
   </si>
   <si>
-    <t>24GM0074</t>
+    <t>24GM00I74</t>
   </si>
 </sst>
 </file>
@@ -6338,7 +6338,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8F7C0C84-C31F-4F27-A331-44A6EB2B65A1}" name="PivotTable4" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{8F7C0C84-C31F-4F27-A331-44A6EB2B65A1}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="T1:X13" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="18">
     <pivotField showAll="0"/>
@@ -6771,21 +6771,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F2A0230-2B50-499C-8AAA-A646BAA6FFC2}">
   <dimension ref="A1:X287"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.85546875" customWidth="1"/>
-    <col min="13" max="13" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="2.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11.88671875" customWidth="1"/>
+    <col min="13" max="13" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="2.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6847,7 +6847,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -6915,7 +6915,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>69</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>69</v>
       </c>
@@ -7042,7 +7042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>69</v>
       </c>
@@ -7104,7 +7104,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>69</v>
       </c>
@@ -7166,7 +7166,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>69</v>
       </c>
@@ -7228,7 +7228,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>69</v>
       </c>
@@ -7290,7 +7290,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>69</v>
       </c>
@@ -7355,7 +7355,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>69</v>
       </c>
@@ -7420,7 +7420,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>69</v>
       </c>
@@ -7488,7 +7488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>69</v>
       </c>
@@ -7553,7 +7553,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>69</v>
       </c>
@@ -7621,7 +7621,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>69</v>
       </c>
@@ -7674,7 +7674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>69</v>
       </c>
@@ -7736,7 +7736,7 @@
         <v>0.995</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:24" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>69</v>
       </c>
@@ -7796,7 +7796,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="17" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>69</v>
       </c>
@@ -7858,7 +7858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -7918,7 +7918,7 @@
         <v>1.002</v>
       </c>
     </row>
-    <row r="19" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>69</v>
       </c>
@@ -7978,7 +7978,7 @@
       </c>
       <c r="V19" s="18"/>
     </row>
-    <row r="20" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -8038,7 +8038,7 @@
       </c>
       <c r="V20" s="18"/>
     </row>
-    <row r="21" spans="1:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -8098,7 +8098,7 @@
       </c>
       <c r="V21" s="18"/>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>69</v>
       </c>
@@ -8151,7 +8151,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>69</v>
       </c>
@@ -8204,7 +8204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -8257,7 +8257,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>69</v>
       </c>
@@ -8310,7 +8310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>69</v>
       </c>
@@ -8363,7 +8363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>69</v>
       </c>
@@ -8416,7 +8416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>69</v>
       </c>
@@ -8469,7 +8469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>69</v>
       </c>
@@ -8522,7 +8522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>69</v>
       </c>
@@ -8575,7 +8575,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>69</v>
       </c>
@@ -8628,7 +8628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>69</v>
       </c>
@@ -8681,7 +8681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>69</v>
       </c>
@@ -8734,7 +8734,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -8787,7 +8787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>69</v>
       </c>
@@ -8840,7 +8840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>69</v>
       </c>
@@ -8893,7 +8893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>69</v>
       </c>
@@ -8946,7 +8946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>69</v>
       </c>
@@ -8999,7 +8999,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>69</v>
       </c>
@@ -9052,7 +9052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>69</v>
       </c>
@@ -9105,7 +9105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>69</v>
       </c>
@@ -9158,7 +9158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>69</v>
       </c>
@@ -9211,7 +9211,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>69</v>
       </c>
@@ -9264,7 +9264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>69</v>
       </c>
@@ -9317,7 +9317,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>69</v>
       </c>
@@ -9370,7 +9370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>69</v>
       </c>
@@ -9423,7 +9423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>69</v>
       </c>
@@ -9476,7 +9476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>69</v>
       </c>
@@ -9529,7 +9529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>69</v>
       </c>
@@ -9582,7 +9582,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>69</v>
       </c>
@@ -9635,7 +9635,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>69</v>
       </c>
@@ -9688,7 +9688,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>69</v>
       </c>
@@ -9741,7 +9741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>69</v>
       </c>
@@ -9794,7 +9794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>69</v>
       </c>
@@ -9847,7 +9847,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>69</v>
       </c>
@@ -9900,7 +9900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>69</v>
       </c>
@@ -9953,7 +9953,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>69</v>
       </c>
@@ -10006,7 +10006,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>69</v>
       </c>
@@ -10059,7 +10059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>69</v>
       </c>
@@ -10112,7 +10112,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>69</v>
       </c>
@@ -10165,7 +10165,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>69</v>
       </c>
@@ -10218,7 +10218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>69</v>
       </c>
@@ -10271,7 +10271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>69</v>
       </c>
@@ -10324,7 +10324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>69</v>
       </c>
@@ -10377,7 +10377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>69</v>
       </c>
@@ -10430,7 +10430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>69</v>
       </c>
@@ -10483,7 +10483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>69</v>
       </c>
@@ -10536,7 +10536,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>69</v>
       </c>
@@ -10589,7 +10589,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>69</v>
       </c>
@@ -10642,7 +10642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>69</v>
       </c>
@@ -10695,7 +10695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>69</v>
       </c>
@@ -10748,7 +10748,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>69</v>
       </c>
@@ -10801,7 +10801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>69</v>
       </c>
@@ -10854,7 +10854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>69</v>
       </c>
@@ -10907,7 +10907,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>69</v>
       </c>
@@ -10960,7 +10960,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>69</v>
       </c>
@@ -11013,7 +11013,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>69</v>
       </c>
@@ -11066,7 +11066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>69</v>
       </c>
@@ -11119,7 +11119,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>69</v>
       </c>
@@ -11172,7 +11172,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>69</v>
       </c>
@@ -11225,7 +11225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>69</v>
       </c>
@@ -11278,7 +11278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>69</v>
       </c>
@@ -11331,7 +11331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>69</v>
       </c>
@@ -11384,7 +11384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>69</v>
       </c>
@@ -11437,7 +11437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>69</v>
       </c>
@@ -11490,7 +11490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>69</v>
       </c>
@@ -11543,7 +11543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>69</v>
       </c>
@@ -11596,7 +11596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>69</v>
       </c>
@@ -11649,7 +11649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>69</v>
       </c>
@@ -11702,7 +11702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>69</v>
       </c>
@@ -11755,7 +11755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>69</v>
       </c>
@@ -11808,7 +11808,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>69</v>
       </c>
@@ -11861,7 +11861,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>69</v>
       </c>
@@ -11914,7 +11914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>69</v>
       </c>
@@ -11967,7 +11967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>69</v>
       </c>
@@ -12020,7 +12020,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>69</v>
       </c>
@@ -12073,7 +12073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>69</v>
       </c>
@@ -12126,7 +12126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>69</v>
       </c>
@@ -12179,7 +12179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>69</v>
       </c>
@@ -12232,7 +12232,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>69</v>
       </c>
@@ -12285,7 +12285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>69</v>
       </c>
@@ -12338,7 +12338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>69</v>
       </c>
@@ -12391,7 +12391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>69</v>
       </c>
@@ -12444,7 +12444,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>69</v>
       </c>
@@ -12497,7 +12497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>69</v>
       </c>
@@ -12550,7 +12550,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>69</v>
       </c>
@@ -12603,7 +12603,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>69</v>
       </c>
@@ -12656,7 +12656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>69</v>
       </c>
@@ -12709,7 +12709,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>69</v>
       </c>
@@ -12762,7 +12762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>69</v>
       </c>
@@ -12815,7 +12815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>69</v>
       </c>
@@ -12868,7 +12868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>69</v>
       </c>
@@ -12921,7 +12921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>69</v>
       </c>
@@ -12974,7 +12974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>69</v>
       </c>
@@ -13027,7 +13027,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>69</v>
       </c>
@@ -13080,7 +13080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>69</v>
       </c>
@@ -13133,7 +13133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>69</v>
       </c>
@@ -13186,7 +13186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>69</v>
       </c>
@@ -13239,7 +13239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>69</v>
       </c>
@@ -13292,7 +13292,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>69</v>
       </c>
@@ -13345,7 +13345,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>69</v>
       </c>
@@ -13398,7 +13398,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>69</v>
       </c>
@@ -13451,7 +13451,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>69</v>
       </c>
@@ -13504,7 +13504,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>69</v>
       </c>
@@ -13557,7 +13557,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>69</v>
       </c>
@@ -13610,7 +13610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>69</v>
       </c>
@@ -13663,7 +13663,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>69</v>
       </c>
@@ -13716,7 +13716,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>69</v>
       </c>
@@ -13769,7 +13769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>69</v>
       </c>
@@ -13822,7 +13822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>69</v>
       </c>
@@ -13875,7 +13875,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>69</v>
       </c>
@@ -13928,7 +13928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>69</v>
       </c>
@@ -13981,7 +13981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>69</v>
       </c>
@@ -14034,7 +14034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>69</v>
       </c>
@@ -14087,7 +14087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>69</v>
       </c>
@@ -14140,7 +14140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>69</v>
       </c>
@@ -14193,7 +14193,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>69</v>
       </c>
@@ -14246,7 +14246,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>69</v>
       </c>
@@ -14299,7 +14299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>69</v>
       </c>
@@ -14352,7 +14352,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>69</v>
       </c>
@@ -14405,7 +14405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>69</v>
       </c>
@@ -14458,7 +14458,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>69</v>
       </c>
@@ -14511,7 +14511,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>69</v>
       </c>
@@ -14564,7 +14564,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>69</v>
       </c>
@@ -14617,7 +14617,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>69</v>
       </c>
@@ -14670,7 +14670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A146" s="5" t="s">
         <v>69</v>
       </c>
@@ -14680,7 +14680,7 @@
       <c r="C146" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D146" s="5" t="s">
+      <c r="D146" t="s">
         <v>71</v>
       </c>
       <c r="E146" s="5" t="s">
@@ -14723,7 +14723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A147" s="5" t="s">
         <v>69</v>
       </c>
@@ -14733,7 +14733,7 @@
       <c r="C147" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D147" s="5" t="s">
+      <c r="D147" t="s">
         <v>71</v>
       </c>
       <c r="E147" s="5" t="s">
@@ -14776,7 +14776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A148" s="5" t="s">
         <v>69</v>
       </c>
@@ -14786,7 +14786,7 @@
       <c r="C148" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D148" s="5" t="s">
+      <c r="D148" t="s">
         <v>71</v>
       </c>
       <c r="E148" s="5" t="s">
@@ -14829,7 +14829,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:17" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A149" s="5" t="s">
         <v>69</v>
       </c>
@@ -14839,7 +14839,7 @@
       <c r="C149" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="D149" s="5" t="s">
+      <c r="D149" t="s">
         <v>71</v>
       </c>
       <c r="E149" s="5" t="s">
@@ -14882,676 +14882,675 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H150" s="1"/>
       <c r="K150" s="4"/>
       <c r="L150" s="4"/>
       <c r="M150" s="4"/>
       <c r="N150" s="4"/>
     </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H151" s="1"/>
       <c r="K151" s="2"/>
       <c r="L151" s="2"/>
       <c r="M151" s="3"/>
       <c r="N151" s="3"/>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H152" s="1"/>
       <c r="K152" s="4"/>
       <c r="L152" s="4"/>
       <c r="M152" s="4"/>
       <c r="N152" s="4"/>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H153" s="1"/>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H154" s="1"/>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H155" s="1"/>
       <c r="K155" s="2"/>
       <c r="L155" s="2"/>
       <c r="M155" s="3"/>
       <c r="N155" s="3"/>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H156" s="1"/>
       <c r="K156" s="2"/>
       <c r="L156" s="2"/>
       <c r="M156" s="3"/>
       <c r="N156" s="3"/>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H157" s="1"/>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H158" s="1"/>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H159" s="1"/>
       <c r="K159" s="2"/>
       <c r="L159" s="2"/>
       <c r="M159" s="3"/>
       <c r="N159" s="3"/>
     </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H160" s="1"/>
     </row>
-    <row r="161" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="161" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H161" s="1"/>
     </row>
-    <row r="162" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="162" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H162" s="1"/>
       <c r="K162" s="2"/>
       <c r="L162" s="2"/>
       <c r="M162" s="3"/>
       <c r="N162" s="3"/>
     </row>
-    <row r="163" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="163" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H163" s="1"/>
     </row>
-    <row r="164" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="164" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H164" s="1"/>
     </row>
-    <row r="165" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="165" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H165" s="1"/>
     </row>
-    <row r="166" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="166" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H166" s="1"/>
       <c r="K166" s="2"/>
       <c r="L166" s="2"/>
       <c r="M166" s="3"/>
       <c r="N166" s="3"/>
     </row>
-    <row r="167" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="167" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H167" s="1"/>
       <c r="K167" s="2"/>
       <c r="L167" s="2"/>
       <c r="M167" s="3"/>
       <c r="N167" s="3"/>
     </row>
-    <row r="168" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="168" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H168" s="1"/>
       <c r="K168" s="2"/>
       <c r="L168" s="2"/>
       <c r="M168" s="3"/>
       <c r="N168" s="3"/>
     </row>
-    <row r="169" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="169" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H169" s="1"/>
       <c r="K169" s="2"/>
       <c r="L169" s="2"/>
       <c r="M169" s="3"/>
       <c r="N169" s="3"/>
     </row>
-    <row r="170" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="170" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H170" s="1"/>
       <c r="K170" s="2"/>
       <c r="L170" s="2"/>
       <c r="M170" s="3"/>
       <c r="N170" s="3"/>
     </row>
-    <row r="171" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="171" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H171" s="1"/>
       <c r="K171" s="2"/>
       <c r="L171" s="2"/>
       <c r="M171" s="3"/>
       <c r="N171" s="3"/>
     </row>
-    <row r="172" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="172" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H172" s="1"/>
       <c r="K172" s="2"/>
       <c r="L172" s="2"/>
       <c r="M172" s="3"/>
       <c r="N172" s="3"/>
     </row>
-    <row r="173" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="173" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H173" s="1"/>
       <c r="K173" s="2"/>
       <c r="L173" s="2"/>
       <c r="M173" s="3"/>
       <c r="N173" s="3"/>
     </row>
-    <row r="174" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="174" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H174" s="1"/>
       <c r="K174" s="2"/>
       <c r="L174" s="2"/>
       <c r="M174" s="3"/>
       <c r="N174" s="3"/>
     </row>
-    <row r="175" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="175" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H175" s="1"/>
       <c r="K175" s="2"/>
       <c r="L175" s="2"/>
       <c r="M175" s="3"/>
       <c r="N175" s="3"/>
     </row>
-    <row r="176" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="176" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H176" s="1"/>
       <c r="K176" s="2"/>
       <c r="L176" s="2"/>
       <c r="M176" s="3"/>
       <c r="N176" s="3"/>
     </row>
-    <row r="177" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="177" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H177" s="1"/>
       <c r="K177" s="2"/>
       <c r="L177" s="2"/>
       <c r="M177" s="3"/>
       <c r="N177" s="3"/>
     </row>
-    <row r="178" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="178" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H178" s="1"/>
       <c r="K178" s="2"/>
       <c r="L178" s="2"/>
       <c r="M178" s="3"/>
       <c r="N178" s="3"/>
     </row>
-    <row r="179" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="179" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H179" s="1"/>
       <c r="K179" s="2"/>
       <c r="L179" s="2"/>
       <c r="M179" s="3"/>
       <c r="N179" s="3"/>
     </row>
-    <row r="180" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="180" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H180" s="1"/>
       <c r="K180" s="2"/>
       <c r="L180" s="2"/>
       <c r="M180" s="3"/>
       <c r="N180" s="3"/>
     </row>
-    <row r="181" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="181" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H181" s="1"/>
       <c r="K181" s="2"/>
       <c r="L181" s="2"/>
       <c r="M181" s="3"/>
       <c r="N181" s="3"/>
     </row>
-    <row r="182" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="182" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H182" s="1"/>
       <c r="K182" s="2"/>
       <c r="L182" s="2"/>
       <c r="M182" s="3"/>
       <c r="N182" s="3"/>
     </row>
-    <row r="183" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="183" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H183" s="1"/>
       <c r="K183" s="2"/>
       <c r="L183" s="2"/>
       <c r="M183" s="3"/>
       <c r="N183" s="3"/>
     </row>
-    <row r="184" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="H184" s="8"/>
     </row>
-    <row r="185" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="H185" s="8"/>
     </row>
-    <row r="186" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="H186" s="8"/>
     </row>
-    <row r="187" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="H187" s="8"/>
       <c r="K187" s="2"/>
       <c r="L187" s="2"/>
       <c r="M187" s="9"/>
       <c r="N187" s="9"/>
     </row>
-    <row r="188" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="8:14" s="4" customFormat="1" x14ac:dyDescent="0.3">
       <c r="H188" s="8"/>
     </row>
-    <row r="189" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="189" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H189" s="1"/>
       <c r="K189" s="2"/>
       <c r="L189" s="2"/>
       <c r="M189" s="3"/>
       <c r="N189" s="3"/>
     </row>
-    <row r="190" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="190" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H190" s="1"/>
       <c r="K190" s="4"/>
       <c r="L190" s="4"/>
       <c r="M190" s="4"/>
       <c r="N190" s="4"/>
     </row>
-    <row r="191" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="191" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H191" s="1"/>
     </row>
-    <row r="192" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="192" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H192" s="1"/>
     </row>
-    <row r="193" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="193" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H193" s="1"/>
     </row>
-    <row r="194" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="194" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H194" s="1"/>
       <c r="K194" s="4"/>
       <c r="L194" s="4"/>
       <c r="M194" s="4"/>
       <c r="N194" s="4"/>
     </row>
-    <row r="195" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="195" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H195" s="1"/>
       <c r="K195" s="2"/>
       <c r="L195" s="2"/>
       <c r="M195" s="3"/>
       <c r="N195" s="3"/>
     </row>
-    <row r="196" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="196" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H196" s="1"/>
     </row>
-    <row r="197" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="197" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H197" s="1"/>
       <c r="K197" s="2"/>
       <c r="L197" s="2"/>
       <c r="M197" s="3"/>
       <c r="N197" s="3"/>
     </row>
-    <row r="198" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="198" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H198" s="1"/>
       <c r="K198" s="4"/>
       <c r="L198" s="4"/>
       <c r="M198" s="4"/>
       <c r="N198" s="4"/>
     </row>
-    <row r="199" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="199" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H199" s="1"/>
       <c r="K199" s="2"/>
       <c r="L199" s="2"/>
       <c r="M199" s="3"/>
       <c r="N199" s="3"/>
     </row>
-    <row r="200" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="200" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H200" s="1"/>
       <c r="K200" s="4"/>
       <c r="L200" s="4"/>
       <c r="M200" s="4"/>
       <c r="N200" s="4"/>
     </row>
-    <row r="201" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="201" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H201" s="1"/>
     </row>
-    <row r="202" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="202" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H202" s="1"/>
       <c r="K202" s="2"/>
       <c r="L202" s="2"/>
       <c r="M202" s="3"/>
       <c r="N202" s="3"/>
     </row>
-    <row r="203" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="203" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H203" s="1"/>
     </row>
-    <row r="204" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="204" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H204" s="1"/>
     </row>
-    <row r="205" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="205" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H205" s="1"/>
     </row>
-    <row r="206" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="206" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H206" s="1"/>
     </row>
-    <row r="207" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="207" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H207" s="1"/>
     </row>
-    <row r="208" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="208" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H208" s="1"/>
     </row>
-    <row r="209" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="209" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H209" s="1"/>
     </row>
-    <row r="210" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="210" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H210" s="1"/>
       <c r="K210" s="2"/>
       <c r="L210" s="2"/>
       <c r="M210" s="3"/>
       <c r="N210" s="3"/>
     </row>
-    <row r="211" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="211" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H211" s="1"/>
     </row>
-    <row r="212" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="212" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H212" s="1"/>
       <c r="K212" s="4"/>
       <c r="L212" s="4"/>
       <c r="M212" s="4"/>
       <c r="N212" s="4"/>
     </row>
-    <row r="213" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="213" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H213" s="1"/>
       <c r="K213" s="2"/>
       <c r="L213" s="2"/>
       <c r="M213" s="3"/>
       <c r="N213" s="3"/>
     </row>
-    <row r="214" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="214" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H214" s="1"/>
     </row>
-    <row r="215" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="215" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H215" s="1"/>
     </row>
-    <row r="216" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="216" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H216" s="1"/>
     </row>
-    <row r="217" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="217" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H217" s="1"/>
     </row>
-    <row r="218" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="218" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H218" s="1"/>
     </row>
-    <row r="219" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="219" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H219" s="1"/>
     </row>
-    <row r="220" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="220" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H220" s="1"/>
       <c r="K220" s="4"/>
       <c r="L220" s="4"/>
       <c r="M220" s="4"/>
       <c r="N220" s="4"/>
     </row>
-    <row r="221" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="221" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H221" s="1"/>
     </row>
-    <row r="222" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="222" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H222" s="1"/>
       <c r="K222" s="4"/>
       <c r="L222" s="4"/>
       <c r="M222" s="4"/>
       <c r="N222" s="4"/>
     </row>
-    <row r="223" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="223" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H223" s="1"/>
     </row>
-    <row r="224" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="224" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H224" s="1"/>
       <c r="K224" s="4"/>
       <c r="L224" s="4"/>
       <c r="M224" s="4"/>
       <c r="N224" s="4"/>
     </row>
-    <row r="225" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="225" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H225" s="1"/>
       <c r="K225" s="4"/>
       <c r="L225" s="4"/>
       <c r="M225" s="4"/>
       <c r="N225" s="4"/>
     </row>
-    <row r="226" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="226" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H226" s="1"/>
       <c r="K226" s="4"/>
       <c r="L226" s="4"/>
       <c r="M226" s="4"/>
       <c r="N226" s="4"/>
     </row>
-    <row r="227" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="227" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H227" s="1"/>
     </row>
-    <row r="228" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="228" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H228" s="1"/>
     </row>
-    <row r="229" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="229" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H229" s="1"/>
       <c r="K229" s="2"/>
       <c r="L229" s="2"/>
       <c r="M229" s="3"/>
       <c r="N229" s="3"/>
     </row>
-    <row r="230" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="230" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H230" s="1"/>
       <c r="K230" s="4"/>
       <c r="L230" s="4"/>
       <c r="M230" s="4"/>
       <c r="N230" s="4"/>
     </row>
-    <row r="231" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="231" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H231" s="1"/>
       <c r="K231" s="4"/>
       <c r="L231" s="4"/>
       <c r="M231" s="4"/>
       <c r="N231" s="4"/>
     </row>
-    <row r="232" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="232" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H232" s="1"/>
     </row>
-    <row r="233" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="233" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H233" s="1"/>
     </row>
-    <row r="234" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="234" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H234" s="1"/>
       <c r="K234" s="4"/>
       <c r="L234" s="4"/>
       <c r="M234" s="4"/>
       <c r="N234" s="4"/>
     </row>
-    <row r="235" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="235" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H235" s="1"/>
       <c r="K235" s="2"/>
       <c r="L235" s="2"/>
       <c r="M235" s="3"/>
       <c r="N235" s="3"/>
     </row>
-    <row r="236" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="236" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H236" s="1"/>
     </row>
-    <row r="237" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="237" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H237" s="1"/>
     </row>
-    <row r="238" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="238" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H238" s="1"/>
       <c r="K238" s="4"/>
       <c r="L238" s="4"/>
       <c r="M238" s="4"/>
       <c r="N238" s="4"/>
     </row>
-    <row r="239" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="239" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H239" s="1"/>
       <c r="K239" s="2"/>
       <c r="L239" s="2"/>
       <c r="M239" s="3"/>
       <c r="N239" s="3"/>
     </row>
-    <row r="240" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="240" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H240" s="1"/>
       <c r="K240" s="2"/>
       <c r="L240" s="2"/>
       <c r="M240" s="3"/>
       <c r="N240" s="3"/>
     </row>
-    <row r="241" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="241" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H241" s="1"/>
     </row>
-    <row r="242" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="242" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H242" s="1"/>
       <c r="K242" s="2"/>
       <c r="L242" s="2"/>
       <c r="M242" s="3"/>
       <c r="N242" s="3"/>
     </row>
-    <row r="243" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="243" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H243" s="1"/>
     </row>
-    <row r="244" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="244" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H244" s="1"/>
       <c r="K244" s="2"/>
       <c r="L244" s="2"/>
       <c r="M244" s="3"/>
       <c r="N244" s="3"/>
     </row>
-    <row r="245" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="245" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H245" s="1"/>
     </row>
-    <row r="246" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="246" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H246" s="1"/>
     </row>
-    <row r="247" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="247" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H247" s="1"/>
     </row>
-    <row r="248" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="248" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H248" s="1"/>
     </row>
-    <row r="249" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="249" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H249" s="1"/>
       <c r="K249" s="2"/>
       <c r="L249" s="2"/>
       <c r="M249" s="3"/>
       <c r="N249" s="3"/>
     </row>
-    <row r="250" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="250" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H250" s="1"/>
     </row>
-    <row r="251" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="251" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H251" s="1"/>
     </row>
-    <row r="252" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="252" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H252" s="1"/>
     </row>
-    <row r="253" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="253" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H253" s="1"/>
       <c r="K253" s="2"/>
       <c r="L253" s="2"/>
       <c r="M253" s="3"/>
       <c r="N253" s="3"/>
     </row>
-    <row r="254" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="254" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H254" s="1"/>
     </row>
-    <row r="255" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="255" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H255" s="1"/>
       <c r="K255" s="2"/>
       <c r="L255" s="2"/>
       <c r="M255" s="3"/>
       <c r="N255" s="3"/>
     </row>
-    <row r="256" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="256" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H256" s="1"/>
     </row>
-    <row r="257" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="257" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H257" s="1"/>
       <c r="K257" s="2"/>
       <c r="L257" s="2"/>
       <c r="M257" s="3"/>
       <c r="N257" s="3"/>
     </row>
-    <row r="258" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="258" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H258" s="1"/>
       <c r="K258" s="2"/>
       <c r="L258" s="2"/>
       <c r="M258" s="3"/>
       <c r="N258" s="3"/>
     </row>
-    <row r="259" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="259" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H259" s="1"/>
       <c r="K259" s="2"/>
       <c r="L259" s="2"/>
       <c r="M259" s="3"/>
       <c r="N259" s="3"/>
     </row>
-    <row r="260" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="260" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H260" s="1"/>
       <c r="K260" s="2"/>
       <c r="L260" s="2"/>
       <c r="M260" s="3"/>
       <c r="N260" s="3"/>
     </row>
-    <row r="261" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="261" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H261" s="1"/>
       <c r="K261" s="2"/>
       <c r="L261" s="2"/>
       <c r="M261" s="3"/>
       <c r="N261" s="3"/>
     </row>
-    <row r="262" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="262" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H262" s="1"/>
     </row>
-    <row r="263" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="263" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H263" s="1"/>
     </row>
-    <row r="264" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="264" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H264" s="1"/>
     </row>
-    <row r="265" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="265" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H265" s="1"/>
     </row>
-    <row r="266" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="266" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H266" s="1"/>
     </row>
-    <row r="267" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="267" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H267" s="1"/>
     </row>
-    <row r="268" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="268" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H268" s="1"/>
     </row>
-    <row r="269" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="269" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H269" s="1"/>
     </row>
-    <row r="270" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="270" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H270" s="1"/>
     </row>
-    <row r="271" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="271" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H271" s="1"/>
     </row>
-    <row r="272" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="272" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H272" s="1"/>
     </row>
-    <row r="273" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="273" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H273" s="1"/>
     </row>
-    <row r="274" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="274" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H274" s="1"/>
     </row>
-    <row r="275" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="275" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H275" s="1"/>
       <c r="K275" s="2"/>
       <c r="L275" s="2"/>
       <c r="M275" s="3"/>
       <c r="N275" s="3"/>
     </row>
-    <row r="276" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="276" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H276" s="1"/>
     </row>
-    <row r="277" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="277" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H277" s="1"/>
     </row>
-    <row r="278" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="278" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H278" s="1"/>
     </row>
-    <row r="279" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="279" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H279" s="1"/>
     </row>
-    <row r="280" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="280" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H280" s="1"/>
     </row>
-    <row r="281" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="281" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H281" s="1"/>
     </row>
-    <row r="282" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="282" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H282" s="1"/>
     </row>
-    <row r="283" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="283" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H283" s="1"/>
     </row>
-    <row r="284" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="284" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H284" s="1"/>
     </row>
-    <row r="285" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="285" spans="8:14" x14ac:dyDescent="0.3">
       <c r="H285" s="1"/>
     </row>
-    <row r="286" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="286" spans="8:14" x14ac:dyDescent="0.3">
       <c r="K286" s="2"/>
       <c r="L286" s="2"/>
       <c r="M286" s="3"/>
       <c r="N286" s="3"/>
     </row>
-    <row r="287" spans="8:14" x14ac:dyDescent="0.25">
+    <row r="287" spans="8:14" x14ac:dyDescent="0.3">
       <c r="K287" s="2"/>
       <c r="L287" s="2"/>
       <c r="M287" s="3"/>
       <c r="N287" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R149" xr:uid="{1F2A0230-2B50-499C-8AAA-A646BAA6FFC2}"/>
   <mergeCells count="5">
     <mergeCell ref="T15:T16"/>
     <mergeCell ref="T17:T18"/>

</xml_diff>